<commit_message>
min_date on DSSTDTC filtered on DSDECOD equal to INFORMED CONSENT OBTAINED for CG0143
</commit_message>
<xml_diff>
--- a/sdtm_rules/CORE-000370/positive/01/data/unit-test-coreid-CG0143-positive.xlsx
+++ b/sdtm_rules/CORE-000370/positive/01/data/unit-test-coreid-CG0143-positive.xlsx
@@ -622,7 +622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA9"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1705,6 +1705,126 @@
         </is>
       </c>
       <c r="AA9" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>CDISCCORE01</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DM</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>GUARD-CONSENT-UNDATED</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>999000309999</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>2018-05-08T11:20</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2018-08-29T10:35</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2018-05-08T11:20</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2018-08-29T10:35</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>2018-03-06</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2018-09-04</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>2021-02-16</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>9990003</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>1947-12-23</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>70</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>YEARS</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>WHITE</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>NOT HISPANIC OR LATINO</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>IKD</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>IKd</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>IKD</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>IKd</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
@@ -1721,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J32"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3161,6 +3281,81 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>CDISCCORE01</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>GUARD-CONSENT-UNDATED</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>INFORMED CONSENT OBTAINED</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>INFORMED CONSENT OBTAINED</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>PROTOCOL MILESTONE</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2018-03-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>CDISCCORE01</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>DS</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>GUARD-CONSENT-UNDATED</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>2</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>INFORMED CONSENT FOR AMENDMENT ONE OBTAINED</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>INFORMED CONSENT OBTAINED</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>PROTOCOL MILESTONE</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>